<commit_message>
feat(projet): UO type — criticite OIL + KPI po_fermes/critiques/sante/EAC
- OIL : colonne criticite (BASSE/MOYENNE/HAUTE), 10 colonnes
- Moteur : po_fermes, po_critiques (DEF + BIND + PUSH — 8 PUSH, 7 BIND)
- KPI Excel locaux : EAC = consomme + RAF, derive = EAC - vendues,
  Sante = ROUGE si critique ouvert / ORANGE si ouvert / VERT sinon
- Dashboard : cartes Sante, EAC, Derive, Points critiques

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/projet_TrainSystem/L09U1-CFL2400-CLIM.xlsx
+++ b/projet_TrainSystem/L09U1-CFL2400-CLIM.xlsx
@@ -25,8 +25,15 @@
     <definedName name="kpi_avancement">'KPI'!$B$3</definedName>
     <definedName name="kpi_h_conso">'KPI'!$B$4</definedName>
     <definedName name="kpi_po_ouverts">'KPI'!$B$5</definedName>
-    <definedName name="kpi_po_fournisseur">'KPI'!$B$6</definedName>
-    <definedName name="kpi_po_expert">'KPI'!$B$7</definedName>
+    <definedName name="kpi_po_fermes">'KPI'!$B$6</definedName>
+    <definedName name="kpi_po_critiques">'KPI'!$B$7</definedName>
+    <definedName name="kpi_po_fournisseur">'KPI'!$B$8</definedName>
+    <definedName name="kpi_po_expert">'KPI'!$B$9</definedName>
+    <definedName name="kpi_h_vendues">'KPI'!$B$10</definedName>
+    <definedName name="kpi_raf">'KPI'!$B$11</definedName>
+    <definedName name="kpi_eac">'KPI'!$B$12</definedName>
+    <definedName name="kpi_derive">'KPI'!$B$13</definedName>
+    <definedName name="kpi_sante">'KPI'!$B$14</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -264,18 +271,19 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="tbl_oil" displayName="tbl_oil" ref="A1:I4" headerRowCount="1">
-  <autoFilter ref="A1:I4"/>
-  <tableColumns count="9">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="tbl_oil" displayName="tbl_oil" ref="A1:J4" headerRowCount="1">
+  <autoFilter ref="A1:J4"/>
+  <tableColumns count="10">
     <tableColumn id="1" name="id"/>
     <tableColumn id="2" name="titre"/>
     <tableColumn id="3" name="description"/>
     <tableColumn id="4" name="en_action"/>
     <tableColumn id="5" name="domaine"/>
-    <tableColumn id="6" name="statut"/>
-    <tableColumn id="7" name="date_ouverture"/>
-    <tableColumn id="8" name="date_besoin"/>
-    <tableColumn id="9" name="journal"/>
+    <tableColumn id="6" name="criticite"/>
+    <tableColumn id="7" name="statut"/>
+    <tableColumn id="8" name="date_ouverture"/>
+    <tableColumn id="9" name="date_besoin"/>
+    <tableColumn id="10" name="journal"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
 </table>
@@ -722,7 +730,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A40"/>
+  <dimension ref="A1:A46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="95" customWidth="1" min="1" max="1"/>
@@ -839,134 +847,176 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>DEF $po_fournisseur = COMPUTE(COUNT_IF($po_ouv.en_action, "FOURNISSEUR"))</t>
+          <t>DEF $po_fermes = COMPUTE(COUNT_IF($oil.statut, "CLOS"))</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>DEF $po_expert = COMPUTE(COUNT_IF($po_ouv.en_action, "EXPERT"))</t>
-        </is>
-      </c>
-    </row>
-    <row r="21"/>
+          <t>DEF $po_critiques = COMPUTE(COUNT_IF($po_ouv.criticite, "HAUTE"))</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>DEF $po_fournisseur = COMPUTE(COUNT_IF($po_ouv.en_action, "FOURNISSEUR"))</t>
+        </is>
+      </c>
+    </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t># ── Regles de qualite ───────────────────────────────────────</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>VALIDATE $actifs.avancement : RANGE(0, 100)</t>
-        </is>
-      </c>
-    </row>
+          <t>DEF $po_expert = COMPUTE(COUNT_IF($po_ouv.en_action, "EXPERT"))</t>
+        </is>
+      </c>
+    </row>
+    <row r="23"/>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>VALIDATE $act.applicable : IN("OUI", "NON")</t>
+          <t># ── Regles de qualite ───────────────────────────────────────</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>VALIDATE $oil.statut : IN("OUVERT", "CLOS")</t>
-        </is>
-      </c>
-    </row>
-    <row r="26"/>
+          <t>VALIDATE $actifs.avancement : RANGE(0, 100)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>VALIDATE $act.applicable : IN("OUI", "NON")</t>
+        </is>
+      </c>
+    </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t># ── Affichage local (onglet KPI) ────────────────────────────</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>BIND $avancement -&gt; KPI.kpi_avancement</t>
-        </is>
-      </c>
-    </row>
+          <t>VALIDATE $oil.statut : IN("OUVERT", "CLOS")</t>
+        </is>
+      </c>
+    </row>
+    <row r="28"/>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>BIND $h_conso -&gt; KPI.kpi_h_conso</t>
+          <t># ── Affichage local (onglet KPI) ────────────────────────────</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>BIND $po_ouverts -&gt; KPI.kpi_po_ouverts</t>
+          <t>BIND $avancement -&gt; KPI.kpi_avancement</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>BIND $po_fournisseur -&gt; KPI.kpi_po_fournisseur</t>
+          <t>BIND $h_conso -&gt; KPI.kpi_h_conso</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>BIND $po_expert -&gt; KPI.kpi_po_expert</t>
-        </is>
-      </c>
-    </row>
-    <row r="33"/>
+          <t>BIND $po_ouverts -&gt; KPI.kpi_po_ouverts</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>BIND $po_fermes -&gt; KPI.kpi_po_fermes</t>
+        </is>
+      </c>
+    </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t># ── Publication vers l'ecosysteme ───────────────────────────</t>
+          <t>BIND $po_critiques -&gt; KPI.kpi_po_critiques</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>PUSH $avancement -&gt; uo.L09U1-CFL2400-CLIM.avancement</t>
+          <t>BIND $po_fournisseur -&gt; KPI.kpi_po_fournisseur</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>PUSH $h_conso -&gt; uo.L09U1-CFL2400-CLIM.heures_consommees</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>PUSH $po_ouverts -&gt; uo.L09U1-CFL2400-CLIM.po_ouverts</t>
-        </is>
-      </c>
-    </row>
+          <t>BIND $po_expert -&gt; KPI.kpi_po_expert</t>
+        </is>
+      </c>
+    </row>
+    <row r="37"/>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>PUSH $actifs -&gt; uo.L09U1-CFL2400-CLIM.activites</t>
+          <t># ── Publication vers l'ecosysteme ───────────────────────────</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>PUSH $oil -&gt; uo.L09U1-CFL2400-CLIM.points_ouverts</t>
+          <t>PUSH $avancement -&gt; uo.L09U1-CFL2400-CLIM.avancement</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
+        <is>
+          <t>PUSH $h_conso -&gt; uo.L09U1-CFL2400-CLIM.heures_consommees</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>PUSH $po_ouverts -&gt; uo.L09U1-CFL2400-CLIM.po_ouverts</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>PUSH $po_fermes -&gt; uo.L09U1-CFL2400-CLIM.po_fermes</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>PUSH $po_critiques -&gt; uo.L09U1-CFL2400-CLIM.po_critiques</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>PUSH $actifs -&gt; uo.L09U1-CFL2400-CLIM.activites</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>PUSH $oil -&gt; uo.L09U1-CFL2400-CLIM.points_ouverts</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
         <is>
           <t>PUSH $liv -&gt; uo.L09U1-CFL2400-CLIM.livrables</t>
         </is>
@@ -1006,7 +1056,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-06-11T17:52:08</t>
+          <t>2026-06-11T18:28:37</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1016,7 +1066,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>PULL=0 COLLECT=0 PUSH=6 BIND=5 err=0</t>
+          <t>PULL=0 COLLECT=0 PUSH=8 BIND=7 err=0</t>
         </is>
       </c>
     </row>
@@ -1737,7 +1787,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:J4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1745,10 +1795,11 @@
     <col width="44" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="9" customWidth="1" min="6" max="6"/>
-    <col width="13" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="50" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="50" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1779,20 +1830,25 @@
       </c>
       <c r="F1" s="4" t="inlineStr">
         <is>
+          <t>criticite</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
           <t>statut</t>
         </is>
       </c>
-      <c r="G1" s="4" t="inlineStr">
+      <c r="H1" s="4" t="inlineStr">
         <is>
           <t>date_ouverture</t>
         </is>
       </c>
-      <c r="H1" s="4" t="inlineStr">
+      <c r="I1" s="4" t="inlineStr">
         <is>
           <t>date_besoin</t>
         </is>
       </c>
-      <c r="I1" s="4" t="inlineStr">
+      <c r="J1" s="4" t="inlineStr">
         <is>
           <t>journal</t>
         </is>
@@ -1821,20 +1877,25 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
+          <t>MOYENNE</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
           <t>OUVERT</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>2026-06-02</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="I2" s="6" t="inlineStr">
+      <c r="J2" s="6" t="inlineStr">
         <is>
           <t>02/06 : envoi v0.3 au fournisseur</t>
         </is>
@@ -1868,20 +1929,25 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
+          <t>HAUTE</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
           <t>OUVERT</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>2026-06-05</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="I3" s="6" t="inlineStr">
+      <c r="J3" s="6" t="inlineStr">
         <is>
           <t>05/06 : question posee a l'expert FS</t>
         </is>
@@ -1910,26 +1976,34 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
+          <t>BASSE</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
           <t>CLOS</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>2026-05-28</t>
         </is>
       </c>
-      <c r="I4" s="6" t="inlineStr">
+      <c r="J4" s="6" t="inlineStr">
         <is>
           <t>28/05 : demande IT — 30/05 : acces obtenu, point clos</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="2">
+  <dataValidations count="3">
     <dataValidation sqref="D2:D60" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"SE,FOURNISSEUR,EXPERT,AT,CLIENT,AUTRE"</formula1>
     </dataValidation>
     <dataValidation sqref="F2:F60" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"BASSE,MOYENNE,HAUTE"</formula1>
+    </dataValidation>
+    <dataValidation sqref="G2:G60" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"OUVERT,CLOS"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1946,7 +2020,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -2009,7 +2083,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Dont balle chez fournisseur</t>
+          <t>Points fermés</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -2017,14 +2091,14 @@
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>Points OUVERTS avec en_action = FOURNISSEUR</t>
+          <t>Nombre de points OIL au statut CLOS</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Dont balle chez expert</t>
+          <t>Points critiques ouverts</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -2032,39 +2106,117 @@
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>Points OUVERTS avec en_action = EXPERT</t>
+          <t>Points OUVERTS avec criticite = HAUTE</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
+          <t>Dont balle chez fournisseur</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>1</v>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>Points OUVERTS avec en_action = FOURNISSEUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Dont balle chez expert</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>1</v>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>Points OUVERTS avec en_action = EXPERT</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
           <t>Heures vendues</t>
         </is>
       </c>
-      <c r="B8">
+      <c r="B10">
         <f>heures_vendues</f>
         <v/>
       </c>
-      <c r="C8" s="7" t="inlineStr">
+      <c r="C10" s="7" t="inlineStr">
         <is>
           <t>Lu depuis General (formule Excel)</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>Reste à faire total (h)</t>
         </is>
       </c>
-      <c r="B9">
+      <c r="B11">
         <f>SUM(Activites!I2:I40)</f>
         <v/>
       </c>
-      <c r="C9" s="7" t="inlineStr">
+      <c r="C11" s="7" t="inlineStr">
         <is>
           <t>Somme colonne reste_a_faire (formule Excel)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Heures estimées à terminaison (EAC)</t>
+        </is>
+      </c>
+      <c r="B12">
+        <f>kpi_h_conso+kpi_raf</f>
+        <v/>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>EAC = consommé + reste à faire (formule Excel)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Dérive à terminaison (h)</t>
+        </is>
+      </c>
+      <c r="B13">
+        <f>kpi_eac-kpi_h_vendues</f>
+        <v/>
+      </c>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>EAC − heures vendues : &gt;0 = dépassement prévu (formule Excel)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Santé</t>
+        </is>
+      </c>
+      <c r="B14">
+        <f>IF(kpi_po_critiques&gt;0,"ROUGE",IF(kpi_po_ouverts&gt;0,"ORANGE","VERT"))</f>
+        <v/>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>ROUGE si point critique ouvert · ORANGE si point ouvert · VERT sinon (formule Excel)</t>
         </is>
       </c>
     </row>
@@ -2079,7 +2231,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:G13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -2138,8 +2290,48 @@
         <v/>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="7" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>SANTÉ</t>
+        </is>
+      </c>
+      <c r="C8" s="8" t="inlineStr">
+        <is>
+          <t>EAC (h)</t>
+        </is>
+      </c>
+      <c r="E8" s="8" t="inlineStr">
+        <is>
+          <t>DÉRIVE (h)</t>
+        </is>
+      </c>
+      <c r="G8" s="8" t="inlineStr">
+        <is>
+          <t>PTS CRITIQUES</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="9">
+        <f>kpi_sante</f>
+        <v/>
+      </c>
+      <c r="C10" s="9">
+        <f>kpi_eac</f>
+        <v/>
+      </c>
+      <c r="E10" s="9">
+        <f>kpi_derive</f>
+        <v/>
+      </c>
+      <c r="G10" s="9">
+        <f>kpi_po_critiques</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="inlineStr">
         <is>
           <t>Cette feuille est libre : l'ingénieur la customise (elle ne fait que LIRE l'onglet KPI).</t>
         </is>

</xml_diff>

<commit_message>
style(projet): formats numeriques 2 decimales (KPI, colonnes calculees, Dashboard ROUND)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/projet_TrainSystem/L09U1-CFL2400-CLIM.xlsx
+++ b/projet_TrainSystem/L09U1-CFL2400-CLIM.xlsx
@@ -41,9 +41,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="0.0"/>
-  </numFmts>
+  <numFmts count="0"/>
   <fonts count="10">
     <font>
       <name val="Calibri"/>
@@ -120,7 +118,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -128,11 +126,12 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -713,7 +712,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="10" t="inlineStr">
+      <c r="A1" s="11" t="inlineStr">
         <is>
           <t>Organisation projet (statique v1 — renseignée à la création depuis le Catalogue Projets).</t>
         </is>
@@ -744,7 +743,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="11" t="inlineStr">
+      <c r="A2" s="12" t="inlineStr">
         <is>
           <t>instruction</t>
         </is>
@@ -1056,7 +1055,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-06-11T18:28:37</t>
+          <t>2026-06-11T18:31:34</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -2041,7 +2040,7 @@
           <t>Avancement UO (%)</t>
         </is>
       </c>
-      <c r="B3" t="n">
+      <c r="B3" s="5" t="n">
         <v>45</v>
       </c>
       <c r="C3" s="7" t="inlineStr">
@@ -2056,7 +2055,7 @@
           <t>Heures consommées</t>
         </is>
       </c>
-      <c r="B4" t="n">
+      <c r="B4" s="5" t="n">
         <v>59</v>
       </c>
       <c r="C4" s="7" t="inlineStr">
@@ -2071,7 +2070,7 @@
           <t>Points ouverts</t>
         </is>
       </c>
-      <c r="B5" t="n">
+      <c r="B5" s="8" t="n">
         <v>2</v>
       </c>
       <c r="C5" s="7" t="inlineStr">
@@ -2086,7 +2085,7 @@
           <t>Points fermés</t>
         </is>
       </c>
-      <c r="B6" t="n">
+      <c r="B6" s="8" t="n">
         <v>1</v>
       </c>
       <c r="C6" s="7" t="inlineStr">
@@ -2101,7 +2100,7 @@
           <t>Points critiques ouverts</t>
         </is>
       </c>
-      <c r="B7" t="n">
+      <c r="B7" s="8" t="n">
         <v>1</v>
       </c>
       <c r="C7" s="7" t="inlineStr">
@@ -2116,7 +2115,7 @@
           <t>Dont balle chez fournisseur</t>
         </is>
       </c>
-      <c r="B8" t="n">
+      <c r="B8" s="8" t="n">
         <v>1</v>
       </c>
       <c r="C8" s="7" t="inlineStr">
@@ -2131,7 +2130,7 @@
           <t>Dont balle chez expert</t>
         </is>
       </c>
-      <c r="B9" t="n">
+      <c r="B9" s="8" t="n">
         <v>1</v>
       </c>
       <c r="C9" s="7" t="inlineStr">
@@ -2146,7 +2145,7 @@
           <t>Heures vendues</t>
         </is>
       </c>
-      <c r="B10">
+      <c r="B10" s="8">
         <f>heures_vendues</f>
         <v/>
       </c>
@@ -2162,7 +2161,7 @@
           <t>Reste à faire total (h)</t>
         </is>
       </c>
-      <c r="B11">
+      <c r="B11" s="5">
         <f>SUM(Activites!I2:I40)</f>
         <v/>
       </c>
@@ -2178,7 +2177,7 @@
           <t>Heures estimées à terminaison (EAC)</t>
         </is>
       </c>
-      <c r="B12">
+      <c r="B12" s="5">
         <f>kpi_h_conso+kpi_raf</f>
         <v/>
       </c>
@@ -2194,7 +2193,7 @@
           <t>Dérive à terminaison (h)</t>
         </is>
       </c>
-      <c r="B13">
+      <c r="B13" s="5">
         <f>kpi_eac-kpi_h_vendues</f>
         <v/>
       </c>
@@ -2251,81 +2250,81 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="8" t="inlineStr">
+      <c r="A4" s="9" t="inlineStr">
         <is>
           <t>AVANCEMENT UO</t>
         </is>
       </c>
-      <c r="C4" s="8" t="inlineStr">
+      <c r="C4" s="9" t="inlineStr">
         <is>
           <t>HEURES</t>
         </is>
       </c>
-      <c r="E4" s="8" t="inlineStr">
+      <c r="E4" s="9" t="inlineStr">
         <is>
           <t>POINTS OUVERTS</t>
         </is>
       </c>
-      <c r="G4" s="8" t="inlineStr">
+      <c r="G4" s="9" t="inlineStr">
         <is>
           <t>ATTENTE FOURN.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="9">
-        <f>kpi_avancement&amp;" %"</f>
+      <c r="A6" s="10">
+        <f>ROUND(kpi_avancement,2)&amp;" %"</f>
         <v/>
       </c>
-      <c r="C6" s="9">
-        <f>kpi_h_conso&amp;" / "&amp;heures_vendues&amp;" h"</f>
+      <c r="C6" s="10">
+        <f>ROUND(kpi_h_conso,2)&amp;" / "&amp;heures_vendues&amp;" h"</f>
         <v/>
       </c>
-      <c r="E6" s="9">
+      <c r="E6" s="10">
         <f>kpi_po_ouverts</f>
         <v/>
       </c>
-      <c r="G6" s="9">
+      <c r="G6" s="10">
         <f>kpi_po_fournisseur</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="8" t="inlineStr">
+      <c r="A8" s="9" t="inlineStr">
         <is>
           <t>SANTÉ</t>
         </is>
       </c>
-      <c r="C8" s="8" t="inlineStr">
+      <c r="C8" s="9" t="inlineStr">
         <is>
           <t>EAC (h)</t>
         </is>
       </c>
-      <c r="E8" s="8" t="inlineStr">
+      <c r="E8" s="9" t="inlineStr">
         <is>
           <t>DÉRIVE (h)</t>
         </is>
       </c>
-      <c r="G8" s="8" t="inlineStr">
+      <c r="G8" s="9" t="inlineStr">
         <is>
           <t>PTS CRITIQUES</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="9">
+      <c r="A10" s="10">
         <f>kpi_sante</f>
         <v/>
       </c>
-      <c r="C10" s="9">
-        <f>kpi_eac</f>
+      <c r="C10" s="10">
+        <f>ROUND(kpi_eac,2)</f>
         <v/>
       </c>
-      <c r="E10" s="9">
-        <f>kpi_derive</f>
+      <c r="E10" s="10">
+        <f>ROUND(kpi_derive,2)</f>
         <v/>
       </c>
-      <c r="G10" s="9">
+      <c r="G10" s="10">
         <f>kpi_po_critiques</f>
         <v/>
       </c>
@@ -2352,7 +2351,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="10" t="inlineStr">
+      <c r="A1" s="11" t="inlineStr">
         <is>
           <t>Réservé : visualisation planning (formules à migrer depuis le template d'origine).</t>
         </is>

</xml_diff>